<commit_message>
Per-pickup files: Tahoma 8, left/center alignment, tight column widths, no title depot name, unfrozen panes
- Font: Tahoma size 8 throughout (was Calibri 11)
- Alignment: left everywhere except GP22/GP42/GP45/RE22/RE45/
  UT22/UT42/PC22/PC42, which are centered (applies to header,
  data, TOTAL, and summary rows)
- Column widths now autofit to actual content length (header vs.
  longest value), floored at 10, except ORG CUST (26), COMMODITY
  (24), and TRAFFIC ORDER (28) which keep a fixed wide column
- Title banner drops the depot name, keeping just the pickup
  code(s) — e.g. "BKG PENDING   (LCH27)"
- Freeze panes removed (was frozen below the header)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - PAT TERMINAL 1 & 2 (PORT AUTHORITY OF THAILAND).xlsx
+++ b/output/bkg pending - PAT TERMINAL 1 & 2 (PORT AUTHORITY OF THAILAND).xlsx
@@ -34,19 +34,19 @@
       <sz val="13"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Tahoma"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
+      <name val="Tahoma"/>
+      <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Tahoma"/>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="6">
@@ -103,16 +103,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,45 +497,45 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
-    <col width="15" customWidth="1" min="27" max="27"/>
-    <col width="15" customWidth="1" min="28" max="28"/>
-    <col width="15" customWidth="1" min="29" max="29"/>
-    <col width="15" customWidth="1" min="30" max="30"/>
-    <col width="15" customWidth="1" min="31" max="31"/>
-    <col width="15" customWidth="1" min="32" max="32"/>
-    <col width="15" customWidth="1" min="33" max="33"/>
-    <col width="15" customWidth="1" min="34" max="34"/>
+    <col width="89" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="27" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BKG PENDING — PAT TERMINAL 1 &amp; 2 (PORT AUTHORITY OF THAILAND)   (BKK01+BKK04)</t>
+          <t>BKG PENDING   (BKK01+BKK04)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -623,47 +638,47 @@
           <t>COMMON REMARK</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>GP22</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>GP42</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>GP45</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>RE22</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>RE45</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>UT22</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>UT42</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>PC22</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>PC42</t>
         </is>
@@ -730,975 +745,975 @@
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>HASLS22260801208</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>KJT</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>202609222100</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>HKHKG</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">40Hx3 </t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>20260914</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>PILOT CONSOLIDATOR CO., LTD.</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>GENERAL CARGO (CONSOL)</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>CONSOL</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Pickup : 2026-09-14, Return : 2026-09-15 CONSOL</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="4" t="n">
+      <c r="N3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Q3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="4" t="n">
+      <c r="Q3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="X3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="4">
+      <c r="X3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="5">
         <f>SUM(N3:V3)-W3</f>
         <v/>
       </c>
-      <c r="Z3" s="4">
+      <c r="Z3" s="5">
         <f>MAX(0,N3-MAX(0,W3))</f>
         <v/>
       </c>
-      <c r="AA3" s="4">
+      <c r="AA3" s="5">
         <f>MAX(0,O3-MAX(0,W3-SUM(N3:N3)))</f>
         <v/>
       </c>
-      <c r="AB3" s="4">
+      <c r="AB3" s="5">
         <f>MAX(0,P3-MAX(0,W3-SUM(N3:O3)))</f>
         <v/>
       </c>
-      <c r="AC3" s="4">
+      <c r="AC3" s="5">
         <f>MAX(0,Q3-MAX(0,W3-SUM(N3:P3)))</f>
         <v/>
       </c>
-      <c r="AD3" s="4">
+      <c r="AD3" s="5">
         <f>MAX(0,R3-MAX(0,W3-SUM(N3:Q3)))</f>
         <v/>
       </c>
-      <c r="AE3" s="4">
+      <c r="AE3" s="5">
         <f>MAX(0,S3-MAX(0,W3-SUM(N3:R3)))</f>
         <v/>
       </c>
-      <c r="AF3" s="4">
+      <c r="AF3" s="5">
         <f>MAX(0,T3-MAX(0,W3-SUM(N3:S3)))</f>
         <v/>
       </c>
-      <c r="AG3" s="4">
+      <c r="AG3" s="5">
         <f>MAX(0,U3-MAX(0,W3-SUM(N3:T3)))</f>
         <v/>
       </c>
-      <c r="AH3" s="4">
+      <c r="AH3" s="5">
         <f>MAX(0,V3-MAX(0,W3-SUM(N3:U3)))</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="13" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>HASLS22260801441</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>KJT</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>202609222100</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>KRPUS</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">40Hx1 20'x1 </t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>20260910</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>GATEWAY CONTAINER LINE CO., LTD.</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>GENERAL CARGO (CONSOL)</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>CONSOL</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Pickup : 2026-09-10, Return : 2026-09-11 CONSOL</t>
         </is>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="4" t="n">
+      <c r="O4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="4">
+      <c r="Q4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="5">
         <f>SUM(N4:V4)-W4</f>
         <v/>
       </c>
-      <c r="Z4" s="4">
+      <c r="Z4" s="5">
         <f>MAX(0,N4-MAX(0,W4))</f>
         <v/>
       </c>
-      <c r="AA4" s="4">
+      <c r="AA4" s="5">
         <f>MAX(0,O4-MAX(0,W4-SUM(N4:N4)))</f>
         <v/>
       </c>
-      <c r="AB4" s="4">
+      <c r="AB4" s="5">
         <f>MAX(0,P4-MAX(0,W4-SUM(N4:O4)))</f>
         <v/>
       </c>
-      <c r="AC4" s="4">
+      <c r="AC4" s="5">
         <f>MAX(0,Q4-MAX(0,W4-SUM(N4:P4)))</f>
         <v/>
       </c>
-      <c r="AD4" s="4">
+      <c r="AD4" s="5">
         <f>MAX(0,R4-MAX(0,W4-SUM(N4:Q4)))</f>
         <v/>
       </c>
-      <c r="AE4" s="4">
+      <c r="AE4" s="5">
         <f>MAX(0,S4-MAX(0,W4-SUM(N4:R4)))</f>
         <v/>
       </c>
-      <c r="AF4" s="4">
+      <c r="AF4" s="5">
         <f>MAX(0,T4-MAX(0,W4-SUM(N4:S4)))</f>
         <v/>
       </c>
-      <c r="AG4" s="4">
+      <c r="AG4" s="5">
         <f>MAX(0,U4-MAX(0,W4-SUM(N4:T4)))</f>
         <v/>
       </c>
-      <c r="AH4" s="4">
+      <c r="AH4" s="5">
         <f>MAX(0,V4-MAX(0,W4-SUM(N4:U4)))</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="13" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>HASLS22260801996</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>KMGY</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>202609271700</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>HKHKG</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>20260911</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>ACCORD PILOT LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>GENERAL CARGO (CONSOL)</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>CONSOL</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Pickup : 2026-09-11, Return : 2026-09-11 CONSOL 
 [1ST CY DATE : 17/09/2026 W/O RENT]</t>
         </is>
       </c>
-      <c r="N5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="4" t="n">
+      <c r="N5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="4">
+      <c r="Q5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="5">
         <f>SUM(N5:V5)-W5</f>
         <v/>
       </c>
-      <c r="Z5" s="4">
+      <c r="Z5" s="5">
         <f>MAX(0,N5-MAX(0,W5))</f>
         <v/>
       </c>
-      <c r="AA5" s="4">
+      <c r="AA5" s="5">
         <f>MAX(0,O5-MAX(0,W5-SUM(N5:N5)))</f>
         <v/>
       </c>
-      <c r="AB5" s="4">
+      <c r="AB5" s="5">
         <f>MAX(0,P5-MAX(0,W5-SUM(N5:O5)))</f>
         <v/>
       </c>
-      <c r="AC5" s="4">
+      <c r="AC5" s="5">
         <f>MAX(0,Q5-MAX(0,W5-SUM(N5:P5)))</f>
         <v/>
       </c>
-      <c r="AD5" s="4">
+      <c r="AD5" s="5">
         <f>MAX(0,R5-MAX(0,W5-SUM(N5:Q5)))</f>
         <v/>
       </c>
-      <c r="AE5" s="4">
+      <c r="AE5" s="5">
         <f>MAX(0,S5-MAX(0,W5-SUM(N5:R5)))</f>
         <v/>
       </c>
-      <c r="AF5" s="4">
+      <c r="AF5" s="5">
         <f>MAX(0,T5-MAX(0,W5-SUM(N5:S5)))</f>
         <v/>
       </c>
-      <c r="AG5" s="4">
+      <c r="AG5" s="5">
         <f>MAX(0,U5-MAX(0,W5-SUM(N5:T5)))</f>
         <v/>
       </c>
-      <c r="AH5" s="4">
+      <c r="AH5" s="5">
         <f>MAX(0,V5-MAX(0,W5-SUM(N5:U5)))</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="13" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>HASLS22260802251</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>KMTP</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>202609200900</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>HKHKG</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>20260916</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>V.C.E. COMPANY LIMITED</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>TAPIOCA FLOUR</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">STUFFING @PAT (SPORT LIGHT TOWER 2) DD.16/09/26 *CLS TIME CFS DD.16/09/26 - 17:00HRS.* </t>
         </is>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="4">
+      <c r="O6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="5">
         <f>SUM(N6:V6)-W6</f>
         <v/>
       </c>
-      <c r="Z6" s="4">
+      <c r="Z6" s="5">
         <f>MAX(0,N6-MAX(0,W6))</f>
         <v/>
       </c>
-      <c r="AA6" s="4">
+      <c r="AA6" s="5">
         <f>MAX(0,O6-MAX(0,W6-SUM(N6:N6)))</f>
         <v/>
       </c>
-      <c r="AB6" s="4">
+      <c r="AB6" s="5">
         <f>MAX(0,P6-MAX(0,W6-SUM(N6:O6)))</f>
         <v/>
       </c>
-      <c r="AC6" s="4">
+      <c r="AC6" s="5">
         <f>MAX(0,Q6-MAX(0,W6-SUM(N6:P6)))</f>
         <v/>
       </c>
-      <c r="AD6" s="4">
+      <c r="AD6" s="5">
         <f>MAX(0,R6-MAX(0,W6-SUM(N6:Q6)))</f>
         <v/>
       </c>
-      <c r="AE6" s="4">
+      <c r="AE6" s="5">
         <f>MAX(0,S6-MAX(0,W6-SUM(N6:R6)))</f>
         <v/>
       </c>
-      <c r="AF6" s="4">
+      <c r="AF6" s="5">
         <f>MAX(0,T6-MAX(0,W6-SUM(N6:S6)))</f>
         <v/>
       </c>
-      <c r="AG6" s="4">
+      <c r="AG6" s="5">
         <f>MAX(0,U6-MAX(0,W6-SUM(N6:T6)))</f>
         <v/>
       </c>
-      <c r="AH6" s="4">
+      <c r="AH6" s="5">
         <f>MAX(0,V6-MAX(0,W6-SUM(N6:U6)))</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>HASLS22260802589</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>SWMM</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>2609N</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>202609230900</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>VNSGN</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>20260916</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>QUANTERM LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>GENERAL CARGO (CONSOL)</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>CONSOL</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">CY-RTN : 16-17/09/2026 (CONSOL) *EXTEND CLS TIME : 22/09/2026 @17.00* </t>
         </is>
       </c>
-      <c r="N7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="4" t="n">
+      <c r="N7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="4">
+      <c r="Q7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="5">
         <f>SUM(N7:V7)-W7</f>
         <v/>
       </c>
-      <c r="Z7" s="4">
+      <c r="Z7" s="5">
         <f>MAX(0,N7-MAX(0,W7))</f>
         <v/>
       </c>
-      <c r="AA7" s="4">
+      <c r="AA7" s="5">
         <f>MAX(0,O7-MAX(0,W7-SUM(N7:N7)))</f>
         <v/>
       </c>
-      <c r="AB7" s="4">
+      <c r="AB7" s="5">
         <f>MAX(0,P7-MAX(0,W7-SUM(N7:O7)))</f>
         <v/>
       </c>
-      <c r="AC7" s="4">
+      <c r="AC7" s="5">
         <f>MAX(0,Q7-MAX(0,W7-SUM(N7:P7)))</f>
         <v/>
       </c>
-      <c r="AD7" s="4">
+      <c r="AD7" s="5">
         <f>MAX(0,R7-MAX(0,W7-SUM(N7:Q7)))</f>
         <v/>
       </c>
-      <c r="AE7" s="4">
+      <c r="AE7" s="5">
         <f>MAX(0,S7-MAX(0,W7-SUM(N7:R7)))</f>
         <v/>
       </c>
-      <c r="AF7" s="4">
+      <c r="AF7" s="5">
         <f>MAX(0,T7-MAX(0,W7-SUM(N7:S7)))</f>
         <v/>
       </c>
-      <c r="AG7" s="4">
+      <c r="AG7" s="5">
         <f>MAX(0,U7-MAX(0,W7-SUM(N7:T7)))</f>
         <v/>
       </c>
-      <c r="AH7" s="4">
+      <c r="AH7" s="5">
         <f>MAX(0,V7-MAX(0,W7-SUM(N7:U7)))</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>HASLS22260900309</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>KMTP</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>202609200900</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>HKHKG</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">40Hx3 </t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>20260916</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>ECU WORLDWIDE (THAILAND) CO., LTD.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>GENERAL CARGO (CONSOL)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>CONSOL</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Pickup : 2026-09-16, Return : 2026-09-16 CONSOL</t>
         </is>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="4" t="n">
+      <c r="N8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="4" t="n">
+      <c r="Q8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="X8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="4">
+      <c r="X8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="5">
         <f>SUM(N8:V8)-W8</f>
         <v/>
       </c>
-      <c r="Z8" s="4">
+      <c r="Z8" s="5">
         <f>MAX(0,N8-MAX(0,W8))</f>
         <v/>
       </c>
-      <c r="AA8" s="4">
+      <c r="AA8" s="5">
         <f>MAX(0,O8-MAX(0,W8-SUM(N8:N8)))</f>
         <v/>
       </c>
-      <c r="AB8" s="4">
+      <c r="AB8" s="5">
         <f>MAX(0,P8-MAX(0,W8-SUM(N8:O8)))</f>
         <v/>
       </c>
-      <c r="AC8" s="4">
+      <c r="AC8" s="5">
         <f>MAX(0,Q8-MAX(0,W8-SUM(N8:P8)))</f>
         <v/>
       </c>
-      <c r="AD8" s="4">
+      <c r="AD8" s="5">
         <f>MAX(0,R8-MAX(0,W8-SUM(N8:Q8)))</f>
         <v/>
       </c>
-      <c r="AE8" s="4">
+      <c r="AE8" s="5">
         <f>MAX(0,S8-MAX(0,W8-SUM(N8:R8)))</f>
         <v/>
       </c>
-      <c r="AF8" s="4">
+      <c r="AF8" s="5">
         <f>MAX(0,T8-MAX(0,W8-SUM(N8:S8)))</f>
         <v/>
       </c>
-      <c r="AG8" s="4">
+      <c r="AG8" s="5">
         <f>MAX(0,U8-MAX(0,W8-SUM(N8:T8)))</f>
         <v/>
       </c>
-      <c r="AH8" s="4">
+      <c r="AH8" s="5">
         <f>MAX(0,V8-MAX(0,W8-SUM(N8:U8)))</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5">
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="8">
         <f>SUM(N3:N8)</f>
         <v/>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="8">
         <f>SUM(O3:O8)</f>
         <v/>
       </c>
-      <c r="P9" s="5">
+      <c r="P9" s="8">
         <f>SUM(P3:P8)</f>
         <v/>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="8">
         <f>SUM(Q3:Q8)</f>
         <v/>
       </c>
-      <c r="R9" s="5">
+      <c r="R9" s="8">
         <f>SUM(R3:R8)</f>
         <v/>
       </c>
-      <c r="S9" s="5">
+      <c r="S9" s="8">
         <f>SUM(S3:S8)</f>
         <v/>
       </c>
-      <c r="T9" s="5">
+      <c r="T9" s="8">
         <f>SUM(T3:T8)</f>
         <v/>
       </c>
-      <c r="U9" s="5">
+      <c r="U9" s="8">
         <f>SUM(U3:U8)</f>
         <v/>
       </c>
-      <c r="V9" s="5">
+      <c r="V9" s="8">
         <f>SUM(V3:V8)</f>
         <v/>
       </c>
-      <c r="W9" s="5">
+      <c r="W9" s="7">
         <f>SUM(W3:W8)</f>
         <v/>
       </c>
-      <c r="X9" s="5" t="n"/>
-      <c r="Y9" s="5">
+      <c r="X9" s="7" t="n"/>
+      <c r="Y9" s="7">
         <f>SUM(Y3:Y8)</f>
         <v/>
       </c>
-      <c r="Z9" s="5">
+      <c r="Z9" s="7">
         <f>SUM(Z3:Z8)</f>
         <v/>
       </c>
-      <c r="AA9" s="5">
+      <c r="AA9" s="7">
         <f>SUM(AA3:AA8)</f>
         <v/>
       </c>
-      <c r="AB9" s="5">
+      <c r="AB9" s="7">
         <f>SUM(AB3:AB8)</f>
         <v/>
       </c>
-      <c r="AC9" s="5">
+      <c r="AC9" s="7">
         <f>SUM(AC3:AC8)</f>
         <v/>
       </c>
-      <c r="AD9" s="5">
+      <c r="AD9" s="7">
         <f>SUM(AD3:AD8)</f>
         <v/>
       </c>
-      <c r="AE9" s="5">
+      <c r="AE9" s="7">
         <f>SUM(AE3:AE8)</f>
         <v/>
       </c>
-      <c r="AF9" s="5">
+      <c r="AF9" s="7">
         <f>SUM(AF3:AF8)</f>
         <v/>
       </c>
-      <c r="AG9" s="5">
+      <c r="AG9" s="7">
         <f>SUM(AG3:AG8)</f>
         <v/>
       </c>
-      <c r="AH9" s="5">
+      <c r="AH9" s="7">
         <f>SUM(AH3:AH8)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Pickup Name</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Number of Records</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Total Balance</t>
         </is>
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>PAT TERMINAL 1 (PORT AUTHORITY OF THAILAND)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>PAT TERMINAL 2 (PORT AUTHORITY OF THAILAND)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="5" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="15" ht="13" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="7" t="n">
         <v>8</v>
       </c>
     </row>

</xml_diff>